<commit_message>
Refactor: improve multiple project modules
</commit_message>
<xml_diff>
--- a/data/experiments.xlsx
+++ b/data/experiments.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D08D28A-BF4C-49F4-AFA6-C9B046DF6246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85ABB72-F9AA-4BA5-9BC8-98ECF6C4CC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,6 +13,9 @@
     <sheet name="PAIR-COEFF-VALUES" sheetId="3" r:id="rId3"/>
     <sheet name="PAIR-COEFF-RANGES" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SYSTEMS!$A$1:$K$1</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -23,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="35">
   <si>
     <t>EXPERIMENT</t>
   </si>
@@ -119,6 +122,15 @@
   </si>
   <si>
     <t>Angstroms</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>FALSE</t>
   </si>
 </sst>
 </file>
@@ -129,7 +141,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.000_);[Red]\(#,##0.000\)"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -187,6 +199,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -196,7 +216,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -219,11 +239,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -286,6 +334,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,7 +693,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.21875" style="6" bestFit="1" customWidth="1"/>
@@ -656,7 +710,7 @@
     <col min="26" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -684,11 +738,14 @@
       <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="23" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K1" s="24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>25</v>
       </c>
@@ -719,8 +776,11 @@
       <c r="J2" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K2" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
@@ -751,8 +811,11 @@
       <c r="J3" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>25</v>
       </c>
@@ -783,8 +846,11 @@
       <c r="J4" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K4" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>25</v>
       </c>
@@ -815,8 +881,11 @@
       <c r="J5" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K5" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>25</v>
       </c>
@@ -847,8 +916,11 @@
       <c r="J6" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K6" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>25</v>
       </c>
@@ -879,8 +951,11 @@
       <c r="J7" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K7" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>25</v>
       </c>
@@ -911,8 +986,11 @@
       <c r="J8" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K8" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
@@ -943,38 +1021,41 @@
       <c r="J9" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K9" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
     </row>
-    <row r="11" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
     </row>
-    <row r="13" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
     </row>
-    <row r="15" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
     </row>
-    <row r="16" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1005,7 +1086,7 @@
       <c r="C21" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>